<commit_message>
deleted idea folder and added 89% rtp
</commit_message>
<xml_diff>
--- a/RTP_Result_500M.xlsx
+++ b/RTP_Result_500M.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
   <si>
     <t>Metric</t>
   </si>
@@ -119,7 +119,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="15.046875" customWidth="true" bestFit="true"/>
@@ -139,7 +139,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n" s="0">
-        <v>1.0E7</v>
+        <v>5.0E8</v>
       </c>
     </row>
     <row r="3">
@@ -147,7 +147,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n" s="0">
-        <v>1.0E7</v>
+        <v>5.0E8</v>
       </c>
     </row>
     <row r="4">
@@ -155,7 +155,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n" s="0">
-        <v>9241243.0</v>
+        <v>4.29254441E8</v>
       </c>
     </row>
     <row r="5">
@@ -163,7 +163,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n" s="0">
-        <v>92.41243</v>
+        <v>85.85</v>
       </c>
     </row>
     <row r="6">
@@ -171,7 +171,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="n" s="0">
-        <v>15.93085</v>
+        <v>15.93</v>
       </c>
     </row>
     <row r="7">
@@ -179,7 +179,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="n" s="0">
-        <v>8000.0</v>
+        <v>9600.0</v>
       </c>
     </row>
     <row r="8">
@@ -189,13 +189,19 @@
       <c r="B8" t="s" s="1">
         <v>9</v>
       </c>
+      <c r="C8" t="s" s="1">
+        <v>5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
         <v>10</v>
       </c>
       <c r="B9" t="n" s="0">
-        <v>6.057093</v>
+        <v>6.011</v>
+      </c>
+      <c r="C9" t="n" s="0">
+        <v>81.81</v>
       </c>
     </row>
     <row r="10">
@@ -203,7 +209,10 @@
         <v>11</v>
       </c>
       <c r="B10" t="n" s="0">
-        <v>15.206761</v>
+        <v>15.26</v>
+      </c>
+      <c r="C10" t="n" s="0">
+        <v>86.19</v>
       </c>
     </row>
     <row r="11">
@@ -211,7 +220,10 @@
         <v>12</v>
       </c>
       <c r="B11" t="n" s="0">
-        <v>25.929445</v>
+        <v>25.9</v>
+      </c>
+      <c r="C11" t="n" s="0">
+        <v>86.34</v>
       </c>
     </row>
     <row r="12">
@@ -219,7 +231,10 @@
         <v>13</v>
       </c>
       <c r="B12" t="n" s="0">
-        <v>9.669626</v>
+        <v>9.675</v>
+      </c>
+      <c r="C12" t="n" s="0">
+        <v>86.17</v>
       </c>
     </row>
     <row r="13">
@@ -227,7 +242,10 @@
         <v>14</v>
       </c>
       <c r="B13" t="n" s="0">
-        <v>16.135833</v>
+        <v>16.15</v>
+      </c>
+      <c r="C13" t="n" s="0">
+        <v>86.22</v>
       </c>
     </row>
     <row r="14">
@@ -235,7 +253,10 @@
         <v>15</v>
       </c>
       <c r="B14" t="n" s="0">
-        <v>23.655799</v>
+        <v>23.66</v>
+      </c>
+      <c r="C14" t="n" s="0">
+        <v>86.63</v>
       </c>
     </row>
     <row r="15">
@@ -243,7 +264,10 @@
         <v>16</v>
       </c>
       <c r="B15" t="n" s="0">
-        <v>10.252078</v>
+        <v>10.23</v>
+      </c>
+      <c r="C15" t="n" s="0">
+        <v>86.33</v>
       </c>
     </row>
     <row r="16">
@@ -251,7 +275,10 @@
         <v>17</v>
       </c>
       <c r="B16" t="n" s="0">
-        <v>15.304356</v>
+        <v>15.31</v>
+      </c>
+      <c r="C16" t="n" s="0">
+        <v>86.44</v>
       </c>
     </row>
     <row r="17">
@@ -259,7 +286,10 @@
         <v>18</v>
       </c>
       <c r="B17" t="n" s="0">
-        <v>21.144649</v>
+        <v>21.2</v>
+      </c>
+      <c r="C17" t="n" s="0">
+        <v>86.52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RTP fix by changing win amount values in Bigdecimal
</commit_message>
<xml_diff>
--- a/RTP_Result_500M.xlsx
+++ b/RTP_Result_500M.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="37">
   <si>
     <t>Metric</t>
   </si>
@@ -69,6 +69,60 @@
   </si>
   <si>
     <t xml:space="preserve"> Spot 10 </t>
+  </si>
+  <si>
+    <t>Spot2 Breakup</t>
+  </si>
+  <si>
+    <t>hits</t>
+  </si>
+  <si>
+    <t>frequency (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0 </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1 </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2 </t>
+  </si>
+  <si>
+    <t>Spot3 Breakup</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 3 </t>
+  </si>
+  <si>
+    <t>Spot4 Breakup</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 4 </t>
+  </si>
+  <si>
+    <t>Spot5 Breakup</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 5 </t>
+  </si>
+  <si>
+    <t>Spot6 Breakup</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 6 </t>
+  </si>
+  <si>
+    <t>Spot7 Breakup</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 7 </t>
+  </si>
+  <si>
+    <t>Spot8 Breakup</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 8 </t>
   </si>
 </sst>
 </file>
@@ -119,11 +173,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C80"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="15.046875" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="10.68359375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="12.4296875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -139,7 +193,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n" s="0">
-        <v>5.0E8</v>
+        <v>1.0E7</v>
       </c>
     </row>
     <row r="3">
@@ -147,7 +201,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n" s="0">
-        <v>5.0E8</v>
+        <v>1.0E7</v>
       </c>
     </row>
     <row r="4">
@@ -155,7 +209,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n" s="0">
-        <v>4.29254441E8</v>
+        <v>8681472.5</v>
       </c>
     </row>
     <row r="5">
@@ -163,7 +217,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n" s="0">
-        <v>85.85</v>
+        <v>86.81</v>
       </c>
     </row>
     <row r="6">
@@ -171,7 +225,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="n" s="0">
-        <v>15.93</v>
+        <v>15.95</v>
       </c>
     </row>
     <row r="7">
@@ -179,7 +233,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="n" s="0">
-        <v>9600.0</v>
+        <v>4000.0</v>
       </c>
     </row>
     <row r="8">
@@ -198,10 +252,10 @@
         <v>10</v>
       </c>
       <c r="B9" t="n" s="0">
-        <v>6.011</v>
+        <v>6.044</v>
       </c>
       <c r="C9" t="n" s="0">
-        <v>81.81</v>
+        <v>87.17</v>
       </c>
     </row>
     <row r="10">
@@ -209,10 +263,10 @@
         <v>11</v>
       </c>
       <c r="B10" t="n" s="0">
-        <v>15.26</v>
+        <v>15.32</v>
       </c>
       <c r="C10" t="n" s="0">
-        <v>86.19</v>
+        <v>86.77</v>
       </c>
     </row>
     <row r="11">
@@ -220,10 +274,10 @@
         <v>12</v>
       </c>
       <c r="B11" t="n" s="0">
-        <v>25.9</v>
+        <v>25.85</v>
       </c>
       <c r="C11" t="n" s="0">
-        <v>86.34</v>
+        <v>85.89</v>
       </c>
     </row>
     <row r="12">
@@ -231,10 +285,10 @@
         <v>13</v>
       </c>
       <c r="B12" t="n" s="0">
-        <v>9.675</v>
+        <v>9.697</v>
       </c>
       <c r="C12" t="n" s="0">
-        <v>86.17</v>
+        <v>87.09</v>
       </c>
     </row>
     <row r="13">
@@ -242,10 +296,10 @@
         <v>14</v>
       </c>
       <c r="B13" t="n" s="0">
-        <v>16.15</v>
+        <v>16.18</v>
       </c>
       <c r="C13" t="n" s="0">
-        <v>86.22</v>
+        <v>86.24</v>
       </c>
     </row>
     <row r="14">
@@ -253,10 +307,10 @@
         <v>15</v>
       </c>
       <c r="B14" t="n" s="0">
-        <v>23.66</v>
+        <v>23.71</v>
       </c>
       <c r="C14" t="n" s="0">
-        <v>86.63</v>
+        <v>87.31</v>
       </c>
     </row>
     <row r="15">
@@ -264,10 +318,10 @@
         <v>16</v>
       </c>
       <c r="B15" t="n" s="0">
-        <v>10.23</v>
+        <v>10.27</v>
       </c>
       <c r="C15" t="n" s="0">
-        <v>86.33</v>
+        <v>88.26</v>
       </c>
     </row>
     <row r="16">
@@ -275,10 +329,10 @@
         <v>17</v>
       </c>
       <c r="B16" t="n" s="0">
-        <v>15.31</v>
+        <v>15.24</v>
       </c>
       <c r="C16" t="n" s="0">
-        <v>86.44</v>
+        <v>86.15</v>
       </c>
     </row>
     <row r="17">
@@ -286,10 +340,444 @@
         <v>18</v>
       </c>
       <c r="B17" t="n" s="0">
-        <v>21.2</v>
+        <v>21.22</v>
       </c>
       <c r="C17" t="n" s="0">
-        <v>86.52</v>
+        <v>86.46</v>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" t="s" s="1">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="1">
+        <v>20</v>
+      </c>
+      <c r="B20" t="s" s="1">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="B21" t="n" s="0">
+        <v>56.0261</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="B22" t="n" s="0">
+        <v>37.93</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="B23" t="n" s="0">
+        <v>6.044</v>
+      </c>
+    </row>
+    <row r="24"/>
+    <row r="25">
+      <c r="A25" t="s" s="1">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s" s="1">
+        <v>20</v>
+      </c>
+      <c r="B26" t="s" s="1">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="B27" t="n" s="0">
+        <v>41.6383</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="B28" t="n" s="0">
+        <v>43.0449</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="B29" t="n" s="0">
+        <v>13.9178</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B30" t="n" s="0">
+        <v>1.39894</v>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32">
+      <c r="A32" t="s" s="1">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s" s="1">
+        <v>20</v>
+      </c>
+      <c r="B33" t="s" s="1">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="B34" t="n" s="0">
+        <v>30.905</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="B35" t="n" s="0">
+        <v>43.243</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="B36" t="n" s="0">
+        <v>21.2327</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B37" t="n" s="0">
+        <v>4.31197</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="B38" t="n" s="0">
+        <v>0.307296</v>
+      </c>
+    </row>
+    <row r="39"/>
+    <row r="40">
+      <c r="A40" t="s" s="1">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s" s="1">
+        <v>20</v>
+      </c>
+      <c r="B41" t="s" s="1">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="B42" t="n" s="0">
+        <v>22.741</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="B43" t="n" s="0">
+        <v>40.5771</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="B44" t="n" s="0">
+        <v>26.9849</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B45" t="n" s="0">
+        <v>8.41059</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="B46" t="n" s="0">
+        <v>1.22226</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="B47" t="n" s="0">
+        <v>0.064064</v>
+      </c>
+    </row>
+    <row r="48"/>
+    <row r="49">
+      <c r="A49" t="s" s="1">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s" s="1">
+        <v>20</v>
+      </c>
+      <c r="B50" t="s" s="1">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="B51" t="n" s="0">
+        <v>16.6972</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="B52" t="n" s="0">
+        <v>36.3028</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="B53" t="n" s="0">
+        <v>30.8221</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B54" t="n" s="0">
+        <v>12.9944</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="B55" t="n" s="0">
+        <v>2.85753</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="B56" t="n" s="0">
+        <v>0.312497</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B57" t="n" s="0">
+        <v>0.0134891</v>
+      </c>
+    </row>
+    <row r="58"/>
+    <row r="59">
+      <c r="A59" t="s" s="1">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s" s="1">
+        <v>20</v>
+      </c>
+      <c r="B60" t="s" s="1">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="B61" t="n" s="0">
+        <v>12.1567</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="B62" t="n" s="0">
+        <v>31.4867</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="B63" t="n" s="0">
+        <v>32.651</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B64" t="n" s="0">
+        <v>17.5477</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="B65" t="n" s="0">
+        <v>5.20823</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="B66" t="n" s="0">
+        <v>0.871022</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B67" t="n" s="0">
+        <v>0.0759209</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="B68" t="n" s="0">
+        <v>0.00269861</v>
+      </c>
+    </row>
+    <row r="69"/>
+    <row r="70">
+      <c r="A70" t="s" s="1">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="s" s="1">
+        <v>20</v>
+      </c>
+      <c r="B71" t="s" s="1">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="B72" t="n" s="0">
+        <v>8.85572</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="B73" t="n" s="0">
+        <v>26.6215</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="B74" t="n" s="0">
+        <v>32.7958</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B75" t="n" s="0">
+        <v>21.4567</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="B76" t="n" s="0">
+        <v>8.15703</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="B77" t="n" s="0">
+        <v>1.85566</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B78" t="n" s="0">
+        <v>0.240496</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="B79" t="n" s="0">
+        <v>0.0165797</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="B80" t="n" s="0">
+        <v>4.5053528E-4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>